<commit_message>
deploy: main → da08443a91e41118c8772acfc9afd507849744dc
</commit_message>
<xml_diff>
--- a/StructureDefinition-tk-organization.xlsx
+++ b/StructureDefinition-tk-organization.xlsx
@@ -10,13 +10,13 @@
     <sheet name="Elements" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AP$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AP$45</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1414" uniqueCount="336">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1758" uniqueCount="355">
   <si>
     <t>Property</t>
   </si>
@@ -505,7 +505,7 @@
 </t>
   </si>
   <si>
-    <t>Organisationsidentifierare ("logisk adress"), inklusive organisationsnummer</t>
+    <t>Organisationsidentifierare ("logisk adress"): HSA-id (primär) och organisationsnummer</t>
   </si>
   <si>
     <t>Identifier for the organization that is used to identify the organization across multiple disparate systems.</t>
@@ -540,19 +540,26 @@
     <t>./Identifiers</t>
   </si>
   <si>
-    <t>Organization.identifier:organisationsnummer</t>
-  </si>
-  <si>
-    <t>organisationsnummer</t>
-  </si>
-  <si>
-    <t>Identifies this organization  across multiple systems</t>
-  </si>
-  <si>
-    <t>REQ-ORG-2</t>
-  </si>
-  <si>
-    <t>Organization.identifier:organisationsnummer.id</t>
+    <t>Organization.identifier:hsaId</t>
+  </si>
+  <si>
+    <t>hsaId</t>
+  </si>
+  <si>
+    <t>HSA-id (primär identifierare och logisk adress)</t>
+  </si>
+  <si>
+    <t>Organisationens HSA-id. Består av prefixet `SE`, organisationsnumret för den direktanslutna producenten i formatet tio siffror utan bindestreck, samt ett bindestreck och en efterföljande identifierande del. Organisationsnumret i HSA-id:t behöver inte vara organisationsnumret för den organisatoriska enhet som HSA-id:t identifierar. Värdet lagras, returneras och söks exakt som det är skrivet.</t>
+  </si>
+  <si>
+    <t>ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}
+tk-org-hsaid-format:HSA-id består av SE, tio siffror (den direktanslutna producentens organisationsnummer utan bindestreck), ett bindestreck och en efterföljande identifierande del. {value.matches('^SE[0-9]{10}-.+$')}</t>
+  </si>
+  <si>
+    <t>REQ-ORG-6, REQ-ORG-7</t>
+  </si>
+  <si>
+    <t>Organization.identifier:hsaId.id</t>
   </si>
   <si>
     <t>Organization.identifier.id</t>
@@ -574,7 +581,7 @@
     <t>n/a</t>
   </si>
   <si>
-    <t>Organization.identifier:organisationsnummer.extension</t>
+    <t>Organization.identifier:hsaId.extension</t>
   </si>
   <si>
     <t>Organization.identifier.extension</t>
@@ -593,7 +600,7 @@
     <t>Element.extension</t>
   </si>
   <si>
-    <t>Organization.identifier:organisationsnummer.use</t>
+    <t>Organization.identifier:hsaId.use</t>
   </si>
   <si>
     <t>Organization.identifier.use</t>
@@ -623,7 +630,7 @@
     <t>Role.code or implied by context</t>
   </si>
   <si>
-    <t>Organization.identifier:organisationsnummer.type</t>
+    <t>Organization.identifier:hsaId.type</t>
   </si>
   <si>
     <t>Organization.identifier.type</t>
@@ -660,7 +667,7 @@
     <t>CX.5</t>
   </si>
   <si>
-    <t>Organization.identifier:organisationsnummer.system</t>
+    <t>Organization.identifier:hsaId.system</t>
   </si>
   <si>
     <t>Organization.identifier.system</t>
@@ -678,7 +685,7 @@
     <t>There are many sets  of identifiers.  To perform matching of two identifiers, we need to know what set we're dealing with. The system identifies a particular set of unique identifiers.</t>
   </si>
   <si>
-    <t>urn:oid:2.5.4.97</t>
+    <t>urn:oid:1.2.752.29.4.19</t>
   </si>
   <si>
     <t>http://www.acme.com/identifiers/patient</t>
@@ -696,7 +703,7 @@
     <t>./IdentifierType</t>
   </si>
   <si>
-    <t>Organization.identifier:organisationsnummer.value</t>
+    <t>Organization.identifier:hsaId.value</t>
   </si>
   <si>
     <t>Organization.identifier.value</t>
@@ -706,7 +713,7 @@
 </t>
   </si>
   <si>
-    <t>Svenskt organisationsnummer</t>
+    <t>HSA-id, t.ex. SE2321000016-1003</t>
   </si>
   <si>
     <t>The portion of the identifier typically relevant to the user and which is unique within the context of the system.</t>
@@ -734,7 +741,7 @@
     <t>./Value</t>
   </si>
   <si>
-    <t>Organization.identifier:organisationsnummer.period</t>
+    <t>Organization.identifier:hsaId.period</t>
   </si>
   <si>
     <t>Organization.identifier.period</t>
@@ -762,7 +769,7 @@
     <t>./StartDate and ./EndDate</t>
   </si>
   <si>
-    <t>Organization.identifier:organisationsnummer.assigner</t>
+    <t>Organization.identifier:hsaId.assigner</t>
   </si>
   <si>
     <t>Organization.identifier.assigner</t>
@@ -791,6 +798,52 @@
   </si>
   <si>
     <t>./IdentifierIssuingAuthority</t>
+  </si>
+  <si>
+    <t>Organization.identifier:organisationsnummer</t>
+  </si>
+  <si>
+    <t>organisationsnummer</t>
+  </si>
+  <si>
+    <t>Organisationsnummer (anges bara på den juridiska personen)</t>
+  </si>
+  <si>
+    <t>ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}
+tk-org-orgnr-format:Organisationsnummer anges som tio siffror utan bindestreck. {value.matches('^[0-9]{10}$')}</t>
+  </si>
+  <si>
+    <t>REQ-ORG-2, REQ-ORG-8, REQ-WRT-5</t>
+  </si>
+  <si>
+    <t>Organization.identifier:organisationsnummer.id</t>
+  </si>
+  <si>
+    <t>Organization.identifier:organisationsnummer.extension</t>
+  </si>
+  <si>
+    <t>Organization.identifier:organisationsnummer.use</t>
+  </si>
+  <si>
+    <t>Organization.identifier:organisationsnummer.type</t>
+  </si>
+  <si>
+    <t>Organization.identifier:organisationsnummer.system</t>
+  </si>
+  <si>
+    <t>urn:oid:2.5.4.97</t>
+  </si>
+  <si>
+    <t>Organization.identifier:organisationsnummer.value</t>
+  </si>
+  <si>
+    <t>Svenskt organisationsnummer, 10 siffror utan bindestreck (t.ex. 2321000016)</t>
+  </si>
+  <si>
+    <t>Organization.identifier:organisationsnummer.period</t>
+  </si>
+  <si>
+    <t>Organization.identifier:organisationsnummer.assigner</t>
   </si>
   <si>
     <t>Organization.active</t>
@@ -957,13 +1010,20 @@
     <t>Organization.partOf</t>
   </si>
   <si>
-    <t>The organization of which this organization forms a part</t>
+    <t xml:space="preserve">Reference(https://fhir.inera.se/ig/tjanstekatalog/StructureDefinition/tk-organization)
+</t>
+  </si>
+  <si>
+    <t>Överordnad organisation, t.ex. vårdgivaren för en vårdenhet</t>
   </si>
   <si>
     <t>The organization of which this organization forms a part.</t>
   </si>
   <si>
     <t>Need to be able to track the hierarchy of organizations within an organization.</t>
+  </si>
+  <si>
+    <t>REQ-ORG-8</t>
   </si>
   <si>
     <t>.playedBy[classCode=Part].scoper</t>
@@ -1396,7 +1456,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AP36"/>
+  <dimension ref="A1:AP45"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="44.5234375" customWidth="true" bestFit="true"/>
@@ -1409,7 +1469,7 @@
     <col min="8" max="8" width="13.953125" customWidth="true" bestFit="true"/>
     <col min="9" max="9" width="11.3671875" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="64.0390625" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="66.87109375" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>
@@ -1434,7 +1494,7 @@
     <col min="33" max="33" width="9.046875" customWidth="true" bestFit="true" hidden="true"/>
     <col min="34" max="34" width="9.46484375" customWidth="true" bestFit="true"/>
     <col min="35" max="35" width="100.703125" customWidth="true"/>
-    <col min="37" max="37" width="20.72265625" customWidth="true" bestFit="true"/>
+    <col min="37" max="37" width="29.96484375" customWidth="true" bestFit="true"/>
     <col min="38" max="38" width="31.65234375" customWidth="true" bestFit="true"/>
     <col min="39" max="39" width="26.69140625" customWidth="true" bestFit="true"/>
     <col min="40" max="40" width="87.9765625" customWidth="true" bestFit="true"/>
@@ -2661,7 +2721,7 @@
       </c>
       <c r="E11" s="2"/>
       <c r="F11" t="s" s="2">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="G11" t="s" s="2">
         <v>82</v>
@@ -2781,7 +2841,7 @@
       </c>
       <c r="E12" s="2"/>
       <c r="F12" t="s" s="2">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="G12" t="s" s="2">
         <v>92</v>
@@ -2802,7 +2862,7 @@
         <v>167</v>
       </c>
       <c r="M12" t="s" s="2">
-        <v>155</v>
+        <v>168</v>
       </c>
       <c r="N12" s="2"/>
       <c r="O12" t="s" s="2">
@@ -2867,10 +2927,10 @@
         <v>159</v>
       </c>
       <c r="AJ12" t="s" s="2">
-        <v>105</v>
+        <v>169</v>
       </c>
       <c r="AK12" t="s" s="2">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="AL12" t="s" s="2">
         <v>160</v>
@@ -2890,10 +2950,10 @@
     </row>
     <row r="13" hidden="true">
       <c r="A13" t="s" s="2">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B13" t="s" s="2">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" t="s" s="2">
@@ -2919,10 +2979,10 @@
         <v>94</v>
       </c>
       <c r="L13" t="s" s="2">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="M13" t="s" s="2">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="N13" s="2"/>
       <c r="O13" s="2"/>
@@ -2973,7 +3033,7 @@
         <v>80</v>
       </c>
       <c r="AF13" t="s" s="2">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="AG13" t="s" s="2">
         <v>81</v>
@@ -2982,7 +3042,7 @@
         <v>92</v>
       </c>
       <c r="AI13" t="s" s="2">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="AJ13" t="s" s="2">
         <v>80</v>
@@ -2997,7 +3057,7 @@
         <v>80</v>
       </c>
       <c r="AN13" t="s" s="2">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="AO13" t="s" s="2">
         <v>80</v>
@@ -3008,10 +3068,10 @@
     </row>
     <row r="14" hidden="true">
       <c r="A14" t="s" s="2">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" t="s" s="2">
@@ -3040,7 +3100,7 @@
         <v>142</v>
       </c>
       <c r="M14" t="s" s="2">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="N14" t="s" s="2">
         <v>144</v>
@@ -3081,10 +3141,10 @@
         <v>80</v>
       </c>
       <c r="AB14" t="s" s="2">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="AC14" t="s" s="2">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="AD14" t="s" s="2">
         <v>80</v>
@@ -3093,7 +3153,7 @@
         <v>158</v>
       </c>
       <c r="AF14" t="s" s="2">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="AG14" t="s" s="2">
         <v>81</v>
@@ -3117,7 +3177,7 @@
         <v>80</v>
       </c>
       <c r="AN14" t="s" s="2">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="AO14" t="s" s="2">
         <v>80</v>
@@ -3128,10 +3188,10 @@
     </row>
     <row r="15" hidden="true">
       <c r="A15" t="s" s="2">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B15" t="s" s="2">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" t="s" s="2">
@@ -3157,16 +3217,16 @@
         <v>113</v>
       </c>
       <c r="L15" t="s" s="2">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="M15" t="s" s="2">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="N15" t="s" s="2">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="O15" t="s" s="2">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="P15" t="s" s="2">
         <v>80</v>
@@ -3194,10 +3254,10 @@
         <v>117</v>
       </c>
       <c r="Y15" t="s" s="2">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="Z15" t="s" s="2">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="AA15" t="s" s="2">
         <v>80</v>
@@ -3215,7 +3275,7 @@
         <v>80</v>
       </c>
       <c r="AF15" t="s" s="2">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="AG15" t="s" s="2">
         <v>81</v>
@@ -3239,7 +3299,7 @@
         <v>138</v>
       </c>
       <c r="AN15" t="s" s="2">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="AO15" t="s" s="2">
         <v>80</v>
@@ -3250,10 +3310,10 @@
     </row>
     <row r="16" hidden="true">
       <c r="A16" t="s" s="2">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" t="s" s="2">
@@ -3276,19 +3336,19 @@
         <v>93</v>
       </c>
       <c r="K16" t="s" s="2">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="L16" t="s" s="2">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="M16" t="s" s="2">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="N16" t="s" s="2">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="O16" t="s" s="2">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="P16" t="s" s="2">
         <v>80</v>
@@ -3313,13 +3373,13 @@
         <v>80</v>
       </c>
       <c r="X16" t="s" s="2">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="Y16" t="s" s="2">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="Z16" t="s" s="2">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="AA16" t="s" s="2">
         <v>80</v>
@@ -3337,7 +3397,7 @@
         <v>80</v>
       </c>
       <c r="AF16" t="s" s="2">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="AG16" t="s" s="2">
         <v>81</v>
@@ -3358,10 +3418,10 @@
         <v>80</v>
       </c>
       <c r="AM16" t="s" s="2">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="AN16" t="s" s="2">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="AO16" t="s" s="2">
         <v>80</v>
@@ -3372,10 +3432,10 @@
     </row>
     <row r="17" hidden="true">
       <c r="A17" t="s" s="2">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" t="s" s="2">
@@ -3401,16 +3461,16 @@
         <v>107</v>
       </c>
       <c r="L17" t="s" s="2">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="M17" t="s" s="2">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="N17" t="s" s="2">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="O17" t="s" s="2">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="P17" t="s" s="2">
         <v>80</v>
@@ -3420,10 +3480,10 @@
         <v>80</v>
       </c>
       <c r="S17" t="s" s="2">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="T17" t="s" s="2">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="U17" t="s" s="2">
         <v>80</v>
@@ -3459,7 +3519,7 @@
         <v>80</v>
       </c>
       <c r="AF17" t="s" s="2">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="AG17" t="s" s="2">
         <v>81</v>
@@ -3480,24 +3540,24 @@
         <v>80</v>
       </c>
       <c r="AM17" t="s" s="2">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="AN17" t="s" s="2">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="AO17" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AP17" t="s" s="2">
-        <v>215</v>
+        <v>217</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="2">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B18" t="s" s="2">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" t="s" s="2">
@@ -3520,16 +3580,16 @@
         <v>93</v>
       </c>
       <c r="K18" t="s" s="2">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="L18" t="s" s="2">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="M18" t="s" s="2">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="N18" t="s" s="2">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="O18" s="2"/>
       <c r="P18" t="s" s="2">
@@ -3543,7 +3603,7 @@
         <v>80</v>
       </c>
       <c r="T18" t="s" s="2">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="U18" t="s" s="2">
         <v>80</v>
@@ -3579,7 +3639,7 @@
         <v>80</v>
       </c>
       <c r="AF18" t="s" s="2">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="AG18" t="s" s="2">
         <v>81</v>
@@ -3588,7 +3648,7 @@
         <v>92</v>
       </c>
       <c r="AI18" t="s" s="2">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="AJ18" t="s" s="2">
         <v>105</v>
@@ -3600,24 +3660,24 @@
         <v>80</v>
       </c>
       <c r="AM18" t="s" s="2">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="AN18" t="s" s="2">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="AO18" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AP18" t="s" s="2">
-        <v>227</v>
+        <v>229</v>
       </c>
     </row>
     <row r="19" hidden="true">
       <c r="A19" t="s" s="2">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" t="s" s="2">
@@ -3640,13 +3700,13 @@
         <v>93</v>
       </c>
       <c r="K19" t="s" s="2">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="L19" t="s" s="2">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="M19" t="s" s="2">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="N19" s="2"/>
       <c r="O19" s="2"/>
@@ -3697,7 +3757,7 @@
         <v>80</v>
       </c>
       <c r="AF19" t="s" s="2">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="AG19" t="s" s="2">
         <v>81</v>
@@ -3718,24 +3778,24 @@
         <v>80</v>
       </c>
       <c r="AM19" t="s" s="2">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="AN19" t="s" s="2">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="AO19" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AP19" t="s" s="2">
-        <v>236</v>
+        <v>238</v>
       </c>
     </row>
     <row r="20" hidden="true">
       <c r="A20" t="s" s="2">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" t="s" s="2">
@@ -3758,16 +3818,16 @@
         <v>93</v>
       </c>
       <c r="K20" t="s" s="2">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="L20" t="s" s="2">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="M20" t="s" s="2">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="N20" t="s" s="2">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="O20" s="2"/>
       <c r="P20" t="s" s="2">
@@ -3817,7 +3877,7 @@
         <v>80</v>
       </c>
       <c r="AF20" t="s" s="2">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="AG20" t="s" s="2">
         <v>81</v>
@@ -3838,26 +3898,28 @@
         <v>80</v>
       </c>
       <c r="AM20" t="s" s="2">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="AN20" t="s" s="2">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="AO20" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AP20" t="s" s="2">
-        <v>246</v>
+        <v>248</v>
       </c>
     </row>
-    <row r="21" hidden="true">
+    <row r="21">
       <c r="A21" t="s" s="2">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>247</v>
-      </c>
-      <c r="C21" s="2"/>
+        <v>152</v>
+      </c>
+      <c r="C21" t="s" s="2">
+        <v>250</v>
+      </c>
       <c r="D21" t="s" s="2">
         <v>80</v>
       </c>
@@ -3869,117 +3931,113 @@
         <v>92</v>
       </c>
       <c r="H21" t="s" s="2">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="I21" t="s" s="2">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="J21" t="s" s="2">
         <v>93</v>
       </c>
       <c r="K21" t="s" s="2">
-        <v>248</v>
+        <v>153</v>
       </c>
       <c r="L21" t="s" s="2">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="M21" t="s" s="2">
-        <v>250</v>
-      </c>
-      <c r="N21" t="s" s="2">
-        <v>251</v>
-      </c>
+        <v>155</v>
+      </c>
+      <c r="N21" s="2"/>
       <c r="O21" t="s" s="2">
+        <v>156</v>
+      </c>
+      <c r="P21" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q21" s="2"/>
+      <c r="R21" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S21" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T21" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U21" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V21" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W21" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X21" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Y21" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Z21" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA21" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB21" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC21" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD21" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE21" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF21" t="s" s="2">
+        <v>152</v>
+      </c>
+      <c r="AG21" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AH21" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AI21" t="s" s="2">
+        <v>159</v>
+      </c>
+      <c r="AJ21" t="s" s="2">
         <v>252</v>
       </c>
-      <c r="P21" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Q21" t="s" s="2">
+      <c r="AK21" t="s" s="2">
         <v>253</v>
       </c>
-      <c r="R21" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="S21" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="T21" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="U21" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="V21" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="W21" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="X21" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Y21" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="Z21" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AA21" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AB21" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AC21" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AD21" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AE21" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AF21" t="s" s="2">
-        <v>247</v>
-      </c>
-      <c r="AG21" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AH21" t="s" s="2">
-        <v>92</v>
-      </c>
-      <c r="AI21" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AJ21" t="s" s="2">
-        <v>105</v>
-      </c>
-      <c r="AK21" t="s" s="2">
-        <v>80</v>
-      </c>
       <c r="AL21" t="s" s="2">
-        <v>254</v>
+        <v>160</v>
       </c>
       <c r="AM21" t="s" s="2">
-        <v>255</v>
+        <v>161</v>
       </c>
       <c r="AN21" t="s" s="2">
-        <v>256</v>
+        <v>162</v>
       </c>
       <c r="AO21" t="s" s="2">
-        <v>257</v>
+        <v>163</v>
       </c>
       <c r="AP21" t="s" s="2">
-        <v>258</v>
+        <v>164</v>
       </c>
     </row>
     <row r="22" hidden="true">
       <c r="A22" t="s" s="2">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>259</v>
+        <v>172</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
@@ -3990,7 +4048,7 @@
         <v>81</v>
       </c>
       <c r="G22" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="H22" t="s" s="2">
         <v>80</v>
@@ -3999,23 +4057,19 @@
         <v>80</v>
       </c>
       <c r="J22" t="s" s="2">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="K22" t="s" s="2">
-        <v>194</v>
+        <v>94</v>
       </c>
       <c r="L22" t="s" s="2">
-        <v>260</v>
+        <v>173</v>
       </c>
       <c r="M22" t="s" s="2">
-        <v>261</v>
-      </c>
-      <c r="N22" t="s" s="2">
-        <v>262</v>
-      </c>
-      <c r="O22" t="s" s="2">
-        <v>263</v>
-      </c>
+        <v>174</v>
+      </c>
+      <c r="N22" s="2"/>
+      <c r="O22" s="2"/>
       <c r="P22" t="s" s="2">
         <v>80</v>
       </c>
@@ -4039,13 +4093,13 @@
         <v>80</v>
       </c>
       <c r="X22" t="s" s="2">
-        <v>264</v>
+        <v>80</v>
       </c>
       <c r="Y22" t="s" s="2">
-        <v>265</v>
+        <v>80</v>
       </c>
       <c r="Z22" t="s" s="2">
-        <v>266</v>
+        <v>80</v>
       </c>
       <c r="AA22" t="s" s="2">
         <v>80</v>
@@ -4063,81 +4117,79 @@
         <v>80</v>
       </c>
       <c r="AF22" t="s" s="2">
-        <v>259</v>
+        <v>175</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH22" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="AI22" t="s" s="2">
-        <v>80</v>
+        <v>176</v>
       </c>
       <c r="AJ22" t="s" s="2">
-        <v>105</v>
+        <v>80</v>
       </c>
       <c r="AK22" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL22" t="s" s="2">
-        <v>267</v>
+        <v>80</v>
       </c>
       <c r="AM22" t="s" s="2">
-        <v>268</v>
+        <v>80</v>
       </c>
       <c r="AN22" t="s" s="2">
-        <v>269</v>
+        <v>177</v>
       </c>
       <c r="AO22" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AP22" t="s" s="2">
-        <v>175</v>
+        <v>80</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" hidden="true">
       <c r="A23" t="s" s="2">
-        <v>270</v>
+        <v>255</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>270</v>
+        <v>179</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
-        <v>80</v>
+        <v>140</v>
       </c>
       <c r="E23" s="2"/>
       <c r="F23" t="s" s="2">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G23" t="s" s="2">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="H23" t="s" s="2">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="I23" t="s" s="2">
         <v>80</v>
       </c>
       <c r="J23" t="s" s="2">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="K23" t="s" s="2">
-        <v>218</v>
+        <v>141</v>
       </c>
       <c r="L23" t="s" s="2">
-        <v>271</v>
+        <v>142</v>
       </c>
       <c r="M23" t="s" s="2">
-        <v>272</v>
+        <v>180</v>
       </c>
       <c r="N23" t="s" s="2">
-        <v>273</v>
-      </c>
-      <c r="O23" t="s" s="2">
-        <v>274</v>
-      </c>
+        <v>144</v>
+      </c>
+      <c r="O23" s="2"/>
       <c r="P23" t="s" s="2">
         <v>80</v>
       </c>
@@ -4173,57 +4225,57 @@
         <v>80</v>
       </c>
       <c r="AB23" t="s" s="2">
-        <v>80</v>
+        <v>181</v>
       </c>
       <c r="AC23" t="s" s="2">
-        <v>80</v>
+        <v>182</v>
       </c>
       <c r="AD23" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AE23" t="s" s="2">
-        <v>80</v>
+        <v>158</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>270</v>
+        <v>183</v>
       </c>
       <c r="AG23" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH23" t="s" s="2">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="AI23" t="s" s="2">
-        <v>159</v>
+        <v>80</v>
       </c>
       <c r="AJ23" t="s" s="2">
-        <v>105</v>
+        <v>146</v>
       </c>
       <c r="AK23" t="s" s="2">
-        <v>99</v>
+        <v>80</v>
       </c>
       <c r="AL23" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AM23" t="s" s="2">
-        <v>275</v>
+        <v>80</v>
       </c>
       <c r="AN23" t="s" s="2">
-        <v>276</v>
+        <v>177</v>
       </c>
       <c r="AO23" t="s" s="2">
-        <v>277</v>
+        <v>80</v>
       </c>
       <c r="AP23" t="s" s="2">
-        <v>278</v>
+        <v>80</v>
       </c>
     </row>
     <row r="24" hidden="true">
       <c r="A24" t="s" s="2">
-        <v>279</v>
+        <v>256</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>279</v>
+        <v>185</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
@@ -4234,31 +4286,31 @@
         <v>81</v>
       </c>
       <c r="G24" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="H24" t="s" s="2">
         <v>80</v>
       </c>
       <c r="I24" t="s" s="2">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="J24" t="s" s="2">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="K24" t="s" s="2">
-        <v>218</v>
+        <v>113</v>
       </c>
       <c r="L24" t="s" s="2">
-        <v>280</v>
+        <v>186</v>
       </c>
       <c r="M24" t="s" s="2">
-        <v>281</v>
+        <v>187</v>
       </c>
       <c r="N24" t="s" s="2">
-        <v>282</v>
+        <v>188</v>
       </c>
       <c r="O24" t="s" s="2">
-        <v>283</v>
+        <v>189</v>
       </c>
       <c r="P24" t="s" s="2">
         <v>80</v>
@@ -4283,13 +4335,13 @@
         <v>80</v>
       </c>
       <c r="X24" t="s" s="2">
-        <v>80</v>
+        <v>117</v>
       </c>
       <c r="Y24" t="s" s="2">
-        <v>80</v>
+        <v>190</v>
       </c>
       <c r="Z24" t="s" s="2">
-        <v>80</v>
+        <v>191</v>
       </c>
       <c r="AA24" t="s" s="2">
         <v>80</v>
@@ -4307,13 +4359,13 @@
         <v>80</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>279</v>
+        <v>192</v>
       </c>
       <c r="AG24" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH24" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="AI24" t="s" s="2">
         <v>80</v>
@@ -4328,10 +4380,10 @@
         <v>80</v>
       </c>
       <c r="AM24" t="s" s="2">
-        <v>80</v>
+        <v>138</v>
       </c>
       <c r="AN24" t="s" s="2">
-        <v>276</v>
+        <v>193</v>
       </c>
       <c r="AO24" t="s" s="2">
         <v>80</v>
@@ -4342,10 +4394,10 @@
     </row>
     <row r="25" hidden="true">
       <c r="A25" t="s" s="2">
-        <v>284</v>
+        <v>257</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>284</v>
+        <v>195</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
@@ -4368,17 +4420,19 @@
         <v>93</v>
       </c>
       <c r="K25" t="s" s="2">
-        <v>285</v>
+        <v>196</v>
       </c>
       <c r="L25" t="s" s="2">
-        <v>286</v>
+        <v>197</v>
       </c>
       <c r="M25" t="s" s="2">
-        <v>287</v>
-      </c>
-      <c r="N25" s="2"/>
+        <v>198</v>
+      </c>
+      <c r="N25" t="s" s="2">
+        <v>199</v>
+      </c>
       <c r="O25" t="s" s="2">
-        <v>288</v>
+        <v>200</v>
       </c>
       <c r="P25" t="s" s="2">
         <v>80</v>
@@ -4403,13 +4457,13 @@
         <v>80</v>
       </c>
       <c r="X25" t="s" s="2">
-        <v>80</v>
+        <v>201</v>
       </c>
       <c r="Y25" t="s" s="2">
-        <v>80</v>
+        <v>202</v>
       </c>
       <c r="Z25" t="s" s="2">
-        <v>80</v>
+        <v>203</v>
       </c>
       <c r="AA25" t="s" s="2">
         <v>80</v>
@@ -4427,7 +4481,7 @@
         <v>80</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>284</v>
+        <v>204</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>81</v>
@@ -4448,10 +4502,10 @@
         <v>80</v>
       </c>
       <c r="AM25" t="s" s="2">
-        <v>80</v>
+        <v>205</v>
       </c>
       <c r="AN25" t="s" s="2">
-        <v>289</v>
+        <v>193</v>
       </c>
       <c r="AO25" t="s" s="2">
         <v>80</v>
@@ -4462,10 +4516,10 @@
     </row>
     <row r="26" hidden="true">
       <c r="A26" t="s" s="2">
-        <v>290</v>
+        <v>258</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>290</v>
+        <v>207</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
@@ -4473,10 +4527,10 @@
       </c>
       <c r="E26" s="2"/>
       <c r="F26" t="s" s="2">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="G26" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="H26" t="s" s="2">
         <v>80</v>
@@ -4485,22 +4539,22 @@
         <v>80</v>
       </c>
       <c r="J26" t="s" s="2">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="K26" t="s" s="2">
-        <v>291</v>
+        <v>107</v>
       </c>
       <c r="L26" t="s" s="2">
-        <v>292</v>
+        <v>208</v>
       </c>
       <c r="M26" t="s" s="2">
-        <v>293</v>
+        <v>209</v>
       </c>
       <c r="N26" t="s" s="2">
-        <v>294</v>
+        <v>210</v>
       </c>
       <c r="O26" t="s" s="2">
-        <v>295</v>
+        <v>211</v>
       </c>
       <c r="P26" t="s" s="2">
         <v>80</v>
@@ -4510,10 +4564,10 @@
         <v>80</v>
       </c>
       <c r="S26" t="s" s="2">
-        <v>80</v>
+        <v>259</v>
       </c>
       <c r="T26" t="s" s="2">
-        <v>80</v>
+        <v>213</v>
       </c>
       <c r="U26" t="s" s="2">
         <v>80</v>
@@ -4549,19 +4603,19 @@
         <v>80</v>
       </c>
       <c r="AF26" t="s" s="2">
-        <v>290</v>
+        <v>214</v>
       </c>
       <c r="AG26" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH26" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="AI26" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ26" t="s" s="2">
-        <v>296</v>
+        <v>105</v>
       </c>
       <c r="AK26" t="s" s="2">
         <v>80</v>
@@ -4570,24 +4624,24 @@
         <v>80</v>
       </c>
       <c r="AM26" t="s" s="2">
-        <v>80</v>
+        <v>215</v>
       </c>
       <c r="AN26" t="s" s="2">
-        <v>297</v>
+        <v>216</v>
       </c>
       <c r="AO26" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AP26" t="s" s="2">
-        <v>80</v>
+        <v>217</v>
       </c>
     </row>
-    <row r="27" hidden="true">
+    <row r="27">
       <c r="A27" t="s" s="2">
-        <v>298</v>
+        <v>260</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>298</v>
+        <v>219</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
@@ -4595,13 +4649,13 @@
       </c>
       <c r="E27" s="2"/>
       <c r="F27" t="s" s="2">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="G27" t="s" s="2">
         <v>92</v>
       </c>
       <c r="H27" t="s" s="2">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="I27" t="s" s="2">
         <v>80</v>
@@ -4610,18 +4664,18 @@
         <v>93</v>
       </c>
       <c r="K27" t="s" s="2">
-        <v>239</v>
+        <v>220</v>
       </c>
       <c r="L27" t="s" s="2">
-        <v>299</v>
+        <v>261</v>
       </c>
       <c r="M27" t="s" s="2">
-        <v>300</v>
-      </c>
-      <c r="N27" s="2"/>
-      <c r="O27" t="s" s="2">
-        <v>301</v>
-      </c>
+        <v>222</v>
+      </c>
+      <c r="N27" t="s" s="2">
+        <v>223</v>
+      </c>
+      <c r="O27" s="2"/>
       <c r="P27" t="s" s="2">
         <v>80</v>
       </c>
@@ -4633,7 +4687,7 @@
         <v>80</v>
       </c>
       <c r="T27" t="s" s="2">
-        <v>80</v>
+        <v>224</v>
       </c>
       <c r="U27" t="s" s="2">
         <v>80</v>
@@ -4669,7 +4723,7 @@
         <v>80</v>
       </c>
       <c r="AF27" t="s" s="2">
-        <v>298</v>
+        <v>225</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>81</v>
@@ -4678,7 +4732,7 @@
         <v>92</v>
       </c>
       <c r="AI27" t="s" s="2">
-        <v>80</v>
+        <v>226</v>
       </c>
       <c r="AJ27" t="s" s="2">
         <v>105</v>
@@ -4690,24 +4744,24 @@
         <v>80</v>
       </c>
       <c r="AM27" t="s" s="2">
-        <v>255</v>
+        <v>227</v>
       </c>
       <c r="AN27" t="s" s="2">
-        <v>302</v>
+        <v>228</v>
       </c>
       <c r="AO27" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AP27" t="s" s="2">
-        <v>175</v>
+        <v>229</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" hidden="true">
       <c r="A28" t="s" s="2">
-        <v>303</v>
+        <v>262</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>303</v>
+        <v>231</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -4718,30 +4772,28 @@
         <v>81</v>
       </c>
       <c r="G28" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="H28" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I28" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J28" t="s" s="2">
         <v>93</v>
       </c>
-      <c r="I28" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="J28" t="s" s="2">
-        <v>80</v>
-      </c>
       <c r="K28" t="s" s="2">
-        <v>304</v>
+        <v>232</v>
       </c>
       <c r="L28" t="s" s="2">
-        <v>305</v>
+        <v>233</v>
       </c>
       <c r="M28" t="s" s="2">
-        <v>306</v>
+        <v>234</v>
       </c>
       <c r="N28" s="2"/>
-      <c r="O28" t="s" s="2">
-        <v>307</v>
-      </c>
+      <c r="O28" s="2"/>
       <c r="P28" t="s" s="2">
         <v>80</v>
       </c>
@@ -4789,13 +4841,13 @@
         <v>80</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>303</v>
+        <v>235</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH28" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="AI28" t="s" s="2">
         <v>80</v>
@@ -4804,30 +4856,30 @@
         <v>105</v>
       </c>
       <c r="AK28" t="s" s="2">
-        <v>308</v>
+        <v>80</v>
       </c>
       <c r="AL28" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AM28" t="s" s="2">
-        <v>80</v>
+        <v>236</v>
       </c>
       <c r="AN28" t="s" s="2">
-        <v>175</v>
+        <v>237</v>
       </c>
       <c r="AO28" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AP28" t="s" s="2">
-        <v>80</v>
+        <v>238</v>
       </c>
     </row>
     <row r="29" hidden="true">
       <c r="A29" t="s" s="2">
-        <v>309</v>
+        <v>263</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>309</v>
+        <v>240</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
@@ -4838,7 +4890,7 @@
         <v>81</v>
       </c>
       <c r="G29" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="H29" t="s" s="2">
         <v>80</v>
@@ -4847,18 +4899,20 @@
         <v>80</v>
       </c>
       <c r="J29" t="s" s="2">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="K29" t="s" s="2">
-        <v>310</v>
+        <v>241</v>
       </c>
       <c r="L29" t="s" s="2">
-        <v>311</v>
+        <v>242</v>
       </c>
       <c r="M29" t="s" s="2">
-        <v>312</v>
-      </c>
-      <c r="N29" s="2"/>
+        <v>243</v>
+      </c>
+      <c r="N29" t="s" s="2">
+        <v>244</v>
+      </c>
       <c r="O29" s="2"/>
       <c r="P29" t="s" s="2">
         <v>80</v>
@@ -4907,13 +4961,13 @@
         <v>80</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>309</v>
+        <v>245</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH29" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="AI29" t="s" s="2">
         <v>80</v>
@@ -4928,24 +4982,24 @@
         <v>80</v>
       </c>
       <c r="AM29" t="s" s="2">
-        <v>313</v>
+        <v>246</v>
       </c>
       <c r="AN29" t="s" s="2">
-        <v>175</v>
+        <v>247</v>
       </c>
       <c r="AO29" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AP29" t="s" s="2">
-        <v>80</v>
+        <v>248</v>
       </c>
     </row>
     <row r="30" hidden="true">
       <c r="A30" t="s" s="2">
-        <v>314</v>
+        <v>264</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>314</v>
+        <v>264</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
@@ -4962,26 +5016,32 @@
         <v>80</v>
       </c>
       <c r="I30" t="s" s="2">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="J30" t="s" s="2">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="K30" t="s" s="2">
-        <v>218</v>
+        <v>265</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>171</v>
+        <v>266</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>172</v>
-      </c>
-      <c r="N30" s="2"/>
-      <c r="O30" s="2"/>
+        <v>267</v>
+      </c>
+      <c r="N30" t="s" s="2">
+        <v>268</v>
+      </c>
+      <c r="O30" t="s" s="2">
+        <v>269</v>
+      </c>
       <c r="P30" t="s" s="2">
         <v>80</v>
       </c>
-      <c r="Q30" s="2"/>
+      <c r="Q30" t="s" s="2">
+        <v>270</v>
+      </c>
       <c r="R30" t="s" s="2">
         <v>80</v>
       </c>
@@ -5025,7 +5085,7 @@
         <v>80</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>173</v>
+        <v>264</v>
       </c>
       <c r="AG30" t="s" s="2">
         <v>81</v>
@@ -5034,40 +5094,40 @@
         <v>92</v>
       </c>
       <c r="AI30" t="s" s="2">
-        <v>174</v>
+        <v>80</v>
       </c>
       <c r="AJ30" t="s" s="2">
-        <v>80</v>
+        <v>105</v>
       </c>
       <c r="AK30" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL30" t="s" s="2">
-        <v>80</v>
+        <v>271</v>
       </c>
       <c r="AM30" t="s" s="2">
-        <v>80</v>
+        <v>272</v>
       </c>
       <c r="AN30" t="s" s="2">
-        <v>175</v>
+        <v>273</v>
       </c>
       <c r="AO30" t="s" s="2">
-        <v>80</v>
+        <v>274</v>
       </c>
       <c r="AP30" t="s" s="2">
-        <v>80</v>
+        <v>275</v>
       </c>
     </row>
     <row r="31" hidden="true">
       <c r="A31" t="s" s="2">
-        <v>315</v>
+        <v>276</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>315</v>
+        <v>276</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
-        <v>140</v>
+        <v>80</v>
       </c>
       <c r="E31" s="2"/>
       <c r="F31" t="s" s="2">
@@ -5083,21 +5143,23 @@
         <v>80</v>
       </c>
       <c r="J31" t="s" s="2">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="K31" t="s" s="2">
-        <v>141</v>
+        <v>196</v>
       </c>
       <c r="L31" t="s" s="2">
-        <v>142</v>
+        <v>277</v>
       </c>
       <c r="M31" t="s" s="2">
-        <v>178</v>
+        <v>278</v>
       </c>
       <c r="N31" t="s" s="2">
-        <v>144</v>
-      </c>
-      <c r="O31" s="2"/>
+        <v>279</v>
+      </c>
+      <c r="O31" t="s" s="2">
+        <v>280</v>
+      </c>
       <c r="P31" t="s" s="2">
         <v>80</v>
       </c>
@@ -5121,13 +5183,13 @@
         <v>80</v>
       </c>
       <c r="X31" t="s" s="2">
-        <v>80</v>
+        <v>281</v>
       </c>
       <c r="Y31" t="s" s="2">
-        <v>80</v>
+        <v>282</v>
       </c>
       <c r="Z31" t="s" s="2">
-        <v>80</v>
+        <v>283</v>
       </c>
       <c r="AA31" t="s" s="2">
         <v>80</v>
@@ -5145,7 +5207,7 @@
         <v>80</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>181</v>
+        <v>276</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>81</v>
@@ -5157,68 +5219,68 @@
         <v>80</v>
       </c>
       <c r="AJ31" t="s" s="2">
-        <v>146</v>
+        <v>105</v>
       </c>
       <c r="AK31" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AL31" t="s" s="2">
-        <v>80</v>
+        <v>284</v>
       </c>
       <c r="AM31" t="s" s="2">
-        <v>80</v>
+        <v>285</v>
       </c>
       <c r="AN31" t="s" s="2">
-        <v>175</v>
+        <v>286</v>
       </c>
       <c r="AO31" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AP31" t="s" s="2">
-        <v>80</v>
+        <v>177</v>
       </c>
     </row>
-    <row r="32" hidden="true">
+    <row r="32">
       <c r="A32" t="s" s="2">
-        <v>316</v>
+        <v>287</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>316</v>
+        <v>287</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
-        <v>317</v>
+        <v>80</v>
       </c>
       <c r="E32" s="2"/>
       <c r="F32" t="s" s="2">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="G32" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="H32" t="s" s="2">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="I32" t="s" s="2">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="J32" t="s" s="2">
         <v>93</v>
       </c>
       <c r="K32" t="s" s="2">
-        <v>141</v>
+        <v>220</v>
       </c>
       <c r="L32" t="s" s="2">
-        <v>318</v>
+        <v>288</v>
       </c>
       <c r="M32" t="s" s="2">
-        <v>319</v>
+        <v>289</v>
       </c>
       <c r="N32" t="s" s="2">
-        <v>144</v>
+        <v>290</v>
       </c>
       <c r="O32" t="s" s="2">
-        <v>150</v>
+        <v>291</v>
       </c>
       <c r="P32" t="s" s="2">
         <v>80</v>
@@ -5267,45 +5329,45 @@
         <v>80</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>320</v>
+        <v>287</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH32" t="s" s="2">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="AI32" t="s" s="2">
-        <v>80</v>
+        <v>159</v>
       </c>
       <c r="AJ32" t="s" s="2">
-        <v>146</v>
+        <v>105</v>
       </c>
       <c r="AK32" t="s" s="2">
-        <v>80</v>
+        <v>99</v>
       </c>
       <c r="AL32" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AM32" t="s" s="2">
-        <v>80</v>
+        <v>292</v>
       </c>
       <c r="AN32" t="s" s="2">
-        <v>138</v>
+        <v>293</v>
       </c>
       <c r="AO32" t="s" s="2">
-        <v>80</v>
+        <v>294</v>
       </c>
       <c r="AP32" t="s" s="2">
-        <v>80</v>
+        <v>295</v>
       </c>
     </row>
     <row r="33" hidden="true">
       <c r="A33" t="s" s="2">
-        <v>321</v>
+        <v>296</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>321</v>
+        <v>296</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
@@ -5328,17 +5390,19 @@
         <v>80</v>
       </c>
       <c r="K33" t="s" s="2">
-        <v>153</v>
+        <v>220</v>
       </c>
       <c r="L33" t="s" s="2">
-        <v>322</v>
+        <v>297</v>
       </c>
       <c r="M33" t="s" s="2">
-        <v>323</v>
-      </c>
-      <c r="N33" s="2"/>
+        <v>298</v>
+      </c>
+      <c r="N33" t="s" s="2">
+        <v>299</v>
+      </c>
       <c r="O33" t="s" s="2">
-        <v>324</v>
+        <v>300</v>
       </c>
       <c r="P33" t="s" s="2">
         <v>80</v>
@@ -5387,7 +5451,7 @@
         <v>80</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>321</v>
+        <v>296</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>81</v>
@@ -5411,7 +5475,7 @@
         <v>80</v>
       </c>
       <c r="AN33" t="s" s="2">
-        <v>175</v>
+        <v>293</v>
       </c>
       <c r="AO33" t="s" s="2">
         <v>80</v>
@@ -5422,10 +5486,10 @@
     </row>
     <row r="34" hidden="true">
       <c r="A34" t="s" s="2">
-        <v>325</v>
+        <v>301</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>325</v>
+        <v>301</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
@@ -5433,7 +5497,7 @@
       </c>
       <c r="E34" s="2"/>
       <c r="F34" t="s" s="2">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="G34" t="s" s="2">
         <v>92</v>
@@ -5445,19 +5509,21 @@
         <v>80</v>
       </c>
       <c r="J34" t="s" s="2">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="K34" t="s" s="2">
-        <v>194</v>
+        <v>302</v>
       </c>
       <c r="L34" t="s" s="2">
-        <v>326</v>
+        <v>303</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>327</v>
+        <v>304</v>
       </c>
       <c r="N34" s="2"/>
-      <c r="O34" s="2"/>
+      <c r="O34" t="s" s="2">
+        <v>305</v>
+      </c>
       <c r="P34" t="s" s="2">
         <v>80</v>
       </c>
@@ -5481,10 +5547,10 @@
         <v>80</v>
       </c>
       <c r="X34" t="s" s="2">
-        <v>264</v>
+        <v>80</v>
       </c>
       <c r="Y34" t="s" s="2">
-        <v>328</v>
+        <v>80</v>
       </c>
       <c r="Z34" t="s" s="2">
         <v>80</v>
@@ -5505,10 +5571,10 @@
         <v>80</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>325</v>
+        <v>301</v>
       </c>
       <c r="AG34" t="s" s="2">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="AH34" t="s" s="2">
         <v>92</v>
@@ -5529,7 +5595,7 @@
         <v>80</v>
       </c>
       <c r="AN34" t="s" s="2">
-        <v>175</v>
+        <v>306</v>
       </c>
       <c r="AO34" t="s" s="2">
         <v>80</v>
@@ -5540,10 +5606,10 @@
     </row>
     <row r="35" hidden="true">
       <c r="A35" t="s" s="2">
-        <v>329</v>
+        <v>307</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>329</v>
+        <v>307</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
@@ -5554,7 +5620,7 @@
         <v>81</v>
       </c>
       <c r="G35" t="s" s="2">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="H35" t="s" s="2">
         <v>80</v>
@@ -5566,17 +5632,19 @@
         <v>80</v>
       </c>
       <c r="K35" t="s" s="2">
-        <v>230</v>
+        <v>308</v>
       </c>
       <c r="L35" t="s" s="2">
-        <v>330</v>
+        <v>309</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>331</v>
-      </c>
-      <c r="N35" s="2"/>
+        <v>310</v>
+      </c>
+      <c r="N35" t="s" s="2">
+        <v>311</v>
+      </c>
       <c r="O35" t="s" s="2">
-        <v>332</v>
+        <v>312</v>
       </c>
       <c r="P35" t="s" s="2">
         <v>80</v>
@@ -5625,19 +5693,19 @@
         <v>80</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>329</v>
+        <v>307</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH35" t="s" s="2">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="AI35" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AJ35" t="s" s="2">
-        <v>105</v>
+        <v>313</v>
       </c>
       <c r="AK35" t="s" s="2">
         <v>80</v>
@@ -5649,7 +5717,7 @@
         <v>80</v>
       </c>
       <c r="AN35" t="s" s="2">
-        <v>175</v>
+        <v>314</v>
       </c>
       <c r="AO35" t="s" s="2">
         <v>80</v>
@@ -5658,12 +5726,12 @@
         <v>80</v>
       </c>
     </row>
-    <row r="36" hidden="true">
+    <row r="36">
       <c r="A36" t="s" s="2">
-        <v>333</v>
+        <v>315</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>333</v>
+        <v>315</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
@@ -5677,25 +5745,27 @@
         <v>92</v>
       </c>
       <c r="H36" t="s" s="2">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="I36" t="s" s="2">
         <v>80</v>
       </c>
       <c r="J36" t="s" s="2">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="K36" t="s" s="2">
-        <v>239</v>
+        <v>316</v>
       </c>
       <c r="L36" t="s" s="2">
-        <v>334</v>
+        <v>317</v>
       </c>
       <c r="M36" t="s" s="2">
-        <v>335</v>
+        <v>318</v>
       </c>
       <c r="N36" s="2"/>
-      <c r="O36" s="2"/>
+      <c r="O36" t="s" s="2">
+        <v>319</v>
+      </c>
       <c r="P36" t="s" s="2">
         <v>80</v>
       </c>
@@ -5743,7 +5813,7 @@
         <v>80</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>333</v>
+        <v>315</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>81</v>
@@ -5758,26 +5828,1100 @@
         <v>105</v>
       </c>
       <c r="AK36" t="s" s="2">
-        <v>80</v>
+        <v>320</v>
       </c>
       <c r="AL36" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AM36" t="s" s="2">
-        <v>80</v>
+        <v>272</v>
       </c>
       <c r="AN36" t="s" s="2">
+        <v>321</v>
+      </c>
+      <c r="AO36" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP36" t="s" s="2">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="s" s="2">
+        <v>322</v>
+      </c>
+      <c r="B37" t="s" s="2">
+        <v>322</v>
+      </c>
+      <c r="C37" s="2"/>
+      <c r="D37" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="E37" s="2"/>
+      <c r="F37" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="G37" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="H37" t="s" s="2">
+        <v>93</v>
+      </c>
+      <c r="I37" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J37" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="K37" t="s" s="2">
+        <v>323</v>
+      </c>
+      <c r="L37" t="s" s="2">
+        <v>324</v>
+      </c>
+      <c r="M37" t="s" s="2">
+        <v>325</v>
+      </c>
+      <c r="N37" s="2"/>
+      <c r="O37" t="s" s="2">
+        <v>326</v>
+      </c>
+      <c r="P37" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q37" s="2"/>
+      <c r="R37" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S37" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T37" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U37" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V37" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W37" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X37" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Y37" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Z37" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA37" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB37" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC37" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD37" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE37" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF37" t="s" s="2">
+        <v>322</v>
+      </c>
+      <c r="AG37" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AH37" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AI37" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ37" t="s" s="2">
+        <v>105</v>
+      </c>
+      <c r="AK37" t="s" s="2">
+        <v>327</v>
+      </c>
+      <c r="AL37" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM37" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN37" t="s" s="2">
+        <v>177</v>
+      </c>
+      <c r="AO37" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP37" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="38" hidden="true">
+      <c r="A38" t="s" s="2">
+        <v>328</v>
+      </c>
+      <c r="B38" t="s" s="2">
+        <v>328</v>
+      </c>
+      <c r="C38" s="2"/>
+      <c r="D38" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="E38" s="2"/>
+      <c r="F38" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="G38" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="H38" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I38" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J38" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="K38" t="s" s="2">
+        <v>329</v>
+      </c>
+      <c r="L38" t="s" s="2">
+        <v>330</v>
+      </c>
+      <c r="M38" t="s" s="2">
+        <v>331</v>
+      </c>
+      <c r="N38" s="2"/>
+      <c r="O38" s="2"/>
+      <c r="P38" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q38" s="2"/>
+      <c r="R38" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S38" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T38" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U38" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V38" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W38" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X38" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Y38" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Z38" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA38" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB38" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC38" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD38" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE38" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF38" t="s" s="2">
+        <v>328</v>
+      </c>
+      <c r="AG38" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AH38" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AI38" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ38" t="s" s="2">
+        <v>105</v>
+      </c>
+      <c r="AK38" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL38" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM38" t="s" s="2">
+        <v>332</v>
+      </c>
+      <c r="AN38" t="s" s="2">
+        <v>177</v>
+      </c>
+      <c r="AO38" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP38" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="39" hidden="true">
+      <c r="A39" t="s" s="2">
+        <v>333</v>
+      </c>
+      <c r="B39" t="s" s="2">
+        <v>333</v>
+      </c>
+      <c r="C39" s="2"/>
+      <c r="D39" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="E39" s="2"/>
+      <c r="F39" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="G39" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="H39" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I39" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J39" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="K39" t="s" s="2">
+        <v>220</v>
+      </c>
+      <c r="L39" t="s" s="2">
+        <v>173</v>
+      </c>
+      <c r="M39" t="s" s="2">
+        <v>174</v>
+      </c>
+      <c r="N39" s="2"/>
+      <c r="O39" s="2"/>
+      <c r="P39" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q39" s="2"/>
+      <c r="R39" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S39" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T39" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U39" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V39" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W39" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X39" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Y39" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Z39" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA39" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB39" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC39" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD39" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE39" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF39" t="s" s="2">
         <v>175</v>
       </c>
-      <c r="AO36" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AP36" t="s" s="2">
+      <c r="AG39" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AH39" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="AI39" t="s" s="2">
+        <v>176</v>
+      </c>
+      <c r="AJ39" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AK39" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL39" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM39" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN39" t="s" s="2">
+        <v>177</v>
+      </c>
+      <c r="AO39" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP39" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="40" hidden="true">
+      <c r="A40" t="s" s="2">
+        <v>334</v>
+      </c>
+      <c r="B40" t="s" s="2">
+        <v>334</v>
+      </c>
+      <c r="C40" s="2"/>
+      <c r="D40" t="s" s="2">
+        <v>140</v>
+      </c>
+      <c r="E40" s="2"/>
+      <c r="F40" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="G40" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="H40" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I40" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J40" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="K40" t="s" s="2">
+        <v>141</v>
+      </c>
+      <c r="L40" t="s" s="2">
+        <v>142</v>
+      </c>
+      <c r="M40" t="s" s="2">
+        <v>180</v>
+      </c>
+      <c r="N40" t="s" s="2">
+        <v>144</v>
+      </c>
+      <c r="O40" s="2"/>
+      <c r="P40" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q40" s="2"/>
+      <c r="R40" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S40" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T40" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U40" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V40" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W40" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X40" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Y40" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Z40" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA40" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB40" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC40" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD40" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE40" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF40" t="s" s="2">
+        <v>183</v>
+      </c>
+      <c r="AG40" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AH40" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AI40" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ40" t="s" s="2">
+        <v>146</v>
+      </c>
+      <c r="AK40" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL40" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM40" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN40" t="s" s="2">
+        <v>177</v>
+      </c>
+      <c r="AO40" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP40" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="41" hidden="true">
+      <c r="A41" t="s" s="2">
+        <v>335</v>
+      </c>
+      <c r="B41" t="s" s="2">
+        <v>335</v>
+      </c>
+      <c r="C41" s="2"/>
+      <c r="D41" t="s" s="2">
+        <v>336</v>
+      </c>
+      <c r="E41" s="2"/>
+      <c r="F41" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="G41" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="H41" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I41" t="s" s="2">
+        <v>93</v>
+      </c>
+      <c r="J41" t="s" s="2">
+        <v>93</v>
+      </c>
+      <c r="K41" t="s" s="2">
+        <v>141</v>
+      </c>
+      <c r="L41" t="s" s="2">
+        <v>337</v>
+      </c>
+      <c r="M41" t="s" s="2">
+        <v>338</v>
+      </c>
+      <c r="N41" t="s" s="2">
+        <v>144</v>
+      </c>
+      <c r="O41" t="s" s="2">
+        <v>150</v>
+      </c>
+      <c r="P41" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q41" s="2"/>
+      <c r="R41" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S41" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T41" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U41" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V41" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W41" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X41" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Y41" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Z41" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA41" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB41" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC41" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD41" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE41" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF41" t="s" s="2">
+        <v>339</v>
+      </c>
+      <c r="AG41" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AH41" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AI41" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ41" t="s" s="2">
+        <v>146</v>
+      </c>
+      <c r="AK41" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL41" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM41" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN41" t="s" s="2">
+        <v>138</v>
+      </c>
+      <c r="AO41" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP41" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="42" hidden="true">
+      <c r="A42" t="s" s="2">
+        <v>340</v>
+      </c>
+      <c r="B42" t="s" s="2">
+        <v>340</v>
+      </c>
+      <c r="C42" s="2"/>
+      <c r="D42" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="E42" s="2"/>
+      <c r="F42" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="G42" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="H42" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I42" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J42" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="K42" t="s" s="2">
+        <v>153</v>
+      </c>
+      <c r="L42" t="s" s="2">
+        <v>341</v>
+      </c>
+      <c r="M42" t="s" s="2">
+        <v>342</v>
+      </c>
+      <c r="N42" s="2"/>
+      <c r="O42" t="s" s="2">
+        <v>343</v>
+      </c>
+      <c r="P42" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q42" s="2"/>
+      <c r="R42" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S42" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T42" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U42" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V42" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W42" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X42" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Y42" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Z42" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA42" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB42" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC42" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD42" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE42" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF42" t="s" s="2">
+        <v>340</v>
+      </c>
+      <c r="AG42" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AH42" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AI42" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ42" t="s" s="2">
+        <v>105</v>
+      </c>
+      <c r="AK42" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL42" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM42" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN42" t="s" s="2">
+        <v>177</v>
+      </c>
+      <c r="AO42" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP42" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="43" hidden="true">
+      <c r="A43" t="s" s="2">
+        <v>344</v>
+      </c>
+      <c r="B43" t="s" s="2">
+        <v>344</v>
+      </c>
+      <c r="C43" s="2"/>
+      <c r="D43" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="E43" s="2"/>
+      <c r="F43" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="G43" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="H43" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I43" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J43" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="K43" t="s" s="2">
+        <v>196</v>
+      </c>
+      <c r="L43" t="s" s="2">
+        <v>345</v>
+      </c>
+      <c r="M43" t="s" s="2">
+        <v>346</v>
+      </c>
+      <c r="N43" s="2"/>
+      <c r="O43" s="2"/>
+      <c r="P43" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q43" s="2"/>
+      <c r="R43" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S43" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T43" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U43" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V43" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W43" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X43" t="s" s="2">
+        <v>281</v>
+      </c>
+      <c r="Y43" t="s" s="2">
+        <v>347</v>
+      </c>
+      <c r="Z43" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA43" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB43" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC43" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD43" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE43" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF43" t="s" s="2">
+        <v>344</v>
+      </c>
+      <c r="AG43" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="AH43" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="AI43" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ43" t="s" s="2">
+        <v>105</v>
+      </c>
+      <c r="AK43" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL43" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM43" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN43" t="s" s="2">
+        <v>177</v>
+      </c>
+      <c r="AO43" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP43" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="44" hidden="true">
+      <c r="A44" t="s" s="2">
+        <v>348</v>
+      </c>
+      <c r="B44" t="s" s="2">
+        <v>348</v>
+      </c>
+      <c r="C44" s="2"/>
+      <c r="D44" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="E44" s="2"/>
+      <c r="F44" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="G44" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="H44" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I44" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J44" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="K44" t="s" s="2">
+        <v>232</v>
+      </c>
+      <c r="L44" t="s" s="2">
+        <v>349</v>
+      </c>
+      <c r="M44" t="s" s="2">
+        <v>350</v>
+      </c>
+      <c r="N44" s="2"/>
+      <c r="O44" t="s" s="2">
+        <v>351</v>
+      </c>
+      <c r="P44" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q44" s="2"/>
+      <c r="R44" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S44" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T44" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U44" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V44" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W44" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X44" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Y44" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Z44" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA44" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB44" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC44" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD44" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE44" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF44" t="s" s="2">
+        <v>348</v>
+      </c>
+      <c r="AG44" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AH44" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="AI44" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ44" t="s" s="2">
+        <v>105</v>
+      </c>
+      <c r="AK44" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL44" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM44" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN44" t="s" s="2">
+        <v>177</v>
+      </c>
+      <c r="AO44" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP44" t="s" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="45" hidden="true">
+      <c r="A45" t="s" s="2">
+        <v>352</v>
+      </c>
+      <c r="B45" t="s" s="2">
+        <v>352</v>
+      </c>
+      <c r="C45" s="2"/>
+      <c r="D45" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="E45" s="2"/>
+      <c r="F45" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="G45" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="H45" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="I45" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="J45" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="K45" t="s" s="2">
+        <v>241</v>
+      </c>
+      <c r="L45" t="s" s="2">
+        <v>353</v>
+      </c>
+      <c r="M45" t="s" s="2">
+        <v>354</v>
+      </c>
+      <c r="N45" s="2"/>
+      <c r="O45" s="2"/>
+      <c r="P45" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Q45" s="2"/>
+      <c r="R45" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="S45" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="T45" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="U45" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="V45" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="W45" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="X45" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Y45" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="Z45" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AA45" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AB45" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AC45" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AD45" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AE45" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AF45" t="s" s="2">
+        <v>352</v>
+      </c>
+      <c r="AG45" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AH45" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="AI45" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AJ45" t="s" s="2">
+        <v>105</v>
+      </c>
+      <c r="AK45" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AL45" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AM45" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AN45" t="s" s="2">
+        <v>177</v>
+      </c>
+      <c r="AO45" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AP45" t="s" s="2">
         <v>80</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AP36">
+  <autoFilter ref="A1:AP45">
     <filterColumn colId="7">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
@@ -5787,7 +6931,7 @@
       <filters blank="true"/>
     </filterColumn>
   </autoFilter>
-  <conditionalFormatting sqref="A2:AI35">
+  <conditionalFormatting sqref="A2:AI44">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$G2&lt;&gt;"Y"</formula>
     </cfRule>

</xml_diff>

<commit_message>
deploy: main → 59740965c7605ec24c4a1b51ef3aae7edcd4de2f
</commit_message>
<xml_diff>
--- a/StructureDefinition-tk-organization.xlsx
+++ b/StructureDefinition-tk-organization.xlsx
@@ -549,11 +549,11 @@
     <t>HSA-id (primär identifierare och logisk adress)</t>
   </si>
   <si>
-    <t>Organisationens HSA-id. Består av prefixet `SE`, organisationsnumret för den direktanslutna producenten i formatet tio siffror utan bindestreck, samt ett bindestreck och en efterföljande identifierande del. Organisationsnumret i HSA-id:t behöver inte vara organisationsnumret för den organisatoriska enhet som HSA-id:t identifierar. Värdet lagras, returneras och söks exakt som det är skrivet.</t>
+    <t>Organisationens HSA-id. Enligt HSA:s styrande dokument är ett HSA-id 1–31 tecken ur a–z, A–Z, 0–9 och bindestreck. Vanligen består det av `SE`, den direktanslutna producentens organisationsnummer utan bindestreck, ett bindestreck och en identifierande del (t.ex. `SE2321000016-1003`), men det finns undantag även i produktion. Ingenting får därför härledas ur ett HSA-id, inte heller ett organisationsnummer. Värdet lagras, returneras och söks exakt som det är skrivet.</t>
   </si>
   <si>
     <t>ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}
-tk-org-hsaid-format:HSA-id består av SE, tio siffror (den direktanslutna producentens organisationsnummer utan bindestreck), ett bindestreck och en efterföljande identifierande del. {value.matches('^SE[0-9]{10}-.+$')}</t>
+tk-org-hsaid-format:HSA-id är 1–31 tecken ur a–z, A–Z, 0–9 och bindestreck, enligt HSA:s styrande dokument. {value.matches('^[a-zA-Z0-9-]{1,31}$')}</t>
   </si>
   <si>
     <t>REQ-ORG-6, REQ-ORG-7</t>

</xml_diff>